<commit_message>
fix: progress log z pliku do bazy (agent_bus log) w bi_view_creation_workflow
</commit_message>
<xml_diff>
--- a/solutions/bi/MagNag/MagNag_plan.xlsx
+++ b/solutions/bi/MagNag/MagNag_plan.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dane" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MagNag_plan" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -134,8 +134,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_Dane_1" displayName="T_Dane_1" ref="A1:I79" headerRowCount="1">
-  <autoFilter ref="A1:I79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_MagNag_plan_1" displayName="T_MagNag_plan_1" ref="A1:I92" headerRowCount="1">
+  <autoFilter ref="A1:I92"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Kolejnosc"/>
     <tableColumn id="2" name="CDN_Pole"/>
@@ -440,14 +440,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="39" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="47" customWidth="1" min="8" max="8"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>CASE WHEN 1089 THEN 'Przyjęcie magazynowe' WHEN 1093 THEN 'Awizo dostawy' WHEN 1601 THEN 'Wydanie magazynowe' WHEN 1605 THEN 'Zlecenie wydania z magazynu' ELSE 'Nieznane (' + CAST(MaN_GIDTyp AS VARCHAR) + ')'</t>
+          <t>CASE MaN_GIDTyp WHEN 1089 THEN 'Przyjęcie magazynowe' WHEN 1093 THEN 'Awizo dostawy' WHEN 1601 THEN 'Wydanie magazynowe' WHEN 1605 THEN 'Zlecenie wydania z magazynu' ELSE 'Nieznane (' + CAST(MaN_GIDTyp AS VARCHAR) + ')' END</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CASE WHEN 0 THEN NULL WHEN 1489 THEN 'Przyjęcie zewnętrzne' WHEN 1497 THEN 'Korekta PZ' WHEN 1521 THEN 'Faktura zakupu' WHEN 1529 THEN 'Korekta FZ' WHEN 1603 THEN 'MMW' WHEN 1604 THEN 'MMP' WHEN 1616 THEN 'Rozchód wewnętrzny' WHEN 1617 THEN 'Przychód wewnętrzny' WHEN 1624 THEN 'Korekta RW' WHEN 1625 THEN 'Korekta PW' WHEN 2001 THEN 'Wydanie zewnętrzne' WHEN 2005 THEN 'WZ eksportowe' WHEN 2009 THEN 'Korekta WZ' WHEN 2013 THEN 'Korekta WZE' WHEN 2033 THEN 'Faktura sprzedaży' WHEN 2034 THEN 'Paragon' WHEN 2037 THEN 'Faktura eksportowa' WHEN 2041 THEN 'Korekta FS' WHEN 2042 THEN 'Korekta paragonu' WHEN 960 THEN 'Zamówienie' ELSE 'Nieznane (' + CAST(MaN_ZrdTyp AS VARCHAR) + ')'</t>
+          <t>CASE MaN_ZrdTyp WHEN 0 THEN NULL WHEN 960 THEN 'Zamówienie' WHEN 1489 THEN 'Przyjęcie zewnętrzne' WHEN 1497 THEN 'Korekta PZ' WHEN 1521 THEN 'Faktura zakupu' WHEN 1529 THEN 'Korekta FZ' WHEN 1603 THEN 'Przesunięcie MMW' WHEN 1604 THEN 'Przesunięcie MMP' WHEN 1616 THEN 'Rozchód wewnętrzny' WHEN 1617 THEN 'Przychód wewnętrzny' WHEN 1624 THEN 'Korekta RW' WHEN 1625 THEN 'Korekta PW' WHEN 2001 THEN 'Wydanie zewnętrzne' WHEN 2005 THEN 'WZ eksportowe' WHEN 2009 THEN 'Korekta WZ' WHEN 2013 THEN 'Korekta WZE' WHEN 2033 THEN 'Faktura sprzedaży' WHEN 2034 THEN 'Paragon' WHEN 2037 THEN 'Faktura eksportowa' WHEN 2041 THEN 'Korekta FS' WHEN 2042 THEN 'Korekta paragonu' ELSE 'Nieznane (' + CAST(MaN_ZrdTyp AS VARCHAR) + ')' END</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -748,30 +748,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MaN_ZrdLp</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>ID kolejność dokumentu źródłowego</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Nr_Dokumentu_Zrodlowego</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>JOIN CDN.TraNag (dla typów TraNag) + CDN.ZamNag (typ 960) per MaN_ZrdTyp i MaN_ZrdNumer; format identyczny jak Nr_Dokumentu: SKRÓT-Nr/MM/YY[/Seria]; CASE WHEN 0 THEN NULL</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>JOIN zweryfikowany przez korelację z ID_Dokumentu_Zrodlowego (100%)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -779,17 +781,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MaN_TrMTyp</t>
+          <t>MaN_ZrdLp</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ID typ magazynu transakcji</t>
+          <t>ID kolejność dokumentu źródłowego</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -799,7 +801,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>COUNT DISTINCT=1 (stały=208)</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -810,17 +812,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MaN_TrMFirma</t>
+          <t>MaN_TrMTyp</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ID firma magazynu transakcji</t>
+          <t>ID typ magazynu transakcji</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1464833</t>
+          <t>208</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -830,7 +832,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>GIDFirma — czyste ID systemu</t>
+          <t>COUNT DISTINCT=1 (stały=208)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -841,40 +843,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MaN_TrMNumer</t>
+          <t>MaN_TrMFirma</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ID numer magazynu transakcji</t>
+          <t>ID firma magazynu transakcji</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1, 4, 7, 8, 9, 10</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>ID_Magazynu_Transakcji</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>MaN_TrMNumer</t>
+          <t>1464833</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Dodać Kod_Magazynu_Transakcji (MAG_Kod) + Nazwa_Magazynu_Transakcji (MAG_Nazwa) z CDN.Magazyny</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>GIDFirma — czyste ID systemu</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -882,29 +874,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MaN_TrMLp</t>
+          <t>MaN_TrMNumer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ID kolejność magazynu transakcji</t>
+          <t>ID numer magazynu transakcji</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1, 4, 7, 8, 9, 10</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ID_Magazynu_Transakcji</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>MaN_TrMNumer</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
@@ -913,27 +911,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MaN_TrNTyp</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Typ transakcji</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>8, 9</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Typ_Transakcji</t>
+          <t>Kod_Magazynu_Transakcji</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>CASE MaN_TrNTyp WHEN 8 THEN 'Wydanie' WHEN 9 THEN 'Przyjęcie' ELSE 'Nieznane (' + CAST(MaN_TrNTyp AS VARCHAR) + ')'</t>
+          <t>LEFT JOIN CDN.Magazyny mag_trm ON mag_trm.MAG_GIDNumer = MaN_TrMNumer › mag_trm.MAG_Kod</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -944,7 +934,7 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Wartości 8/9 wynikają z korelacji z GIDTyp (8=WM+ZWM, 9=PM+AWD); dokumentacja opisuje @S3 bez mapowania</t>
+          <t>JOIN 100% (zweryfikowany)</t>
         </is>
       </c>
     </row>
@@ -954,27 +944,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MaN_TrNRok</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Rok transakcji</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2023, 2024</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Rok_Transakcji</t>
+          <t>Nazwa_Magazynu_Transakcji</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>MaN_TrNRok</t>
+          <t>mag_trm.MAG_Nazwa</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -991,35 +973,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MaN_TrNMiesiac</t>
+          <t>MaN_TrMLp</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Miesiąc transakcji</t>
+          <t>ID kolejność magazynu transakcji</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3, 5, 6, 11</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Miesiac_Transakcji</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>MaN_TrNMiesiac</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>GIDLp — czyste ID systemu</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1028,27 +1004,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MaN_TrNSeria</t>
+          <t>MaN_TrNTyp</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Seria dokumentu</t>
+          <t>Typ transakcji</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>ZTHKK, SKR, BUS</t>
+          <t>8, 9</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Seria</t>
+          <t>Typ_Transakcji</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>NULLIF(RTRIM(MaN_TrNSeria), '')</t>
+          <t>CASE MaN_TrNTyp WHEN 8 THEN 'Wydanie' WHEN 9 THEN 'Przyjęcie' ELSE 'Nieznane (' + CAST(MaN_TrNTyp AS VARCHAR) + ')' END</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1059,7 +1035,7 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Część Nr_Dokumentu; zachowana osobno</t>
+          <t>Interpretacja z korelacji: 8=WM+ZWM, 9=PM+AWD; dokumentacja @S3 bez mapowania</t>
         </is>
       </c>
     </row>
@@ -1069,27 +1045,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MaN_TrNNumer</t>
+          <t>MaN_TrNRok</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Numer transakcji</t>
+          <t>Rok transakcji</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1, 2, 3</t>
+          <t>2023, 2024</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Nr_Dokumentu</t>
+          <t>Rok_Transakcji</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CASE MaN_GIDTyp WHEN 1089 THEN 'PM' WHEN 1093 THEN 'AWD' WHEN 1601 THEN 'WM' WHEN 1605 THEN 'ZWM' ELSE '??' END + '-' + CAST(MaN_TrNNumer AS VARCHAR(10)) + '/' + RIGHT('0' + CAST(MaN_TrNMiesiac AS VARCHAR(2)), 2) + '/' + RIGHT(CAST(MaN_TrNRok AS VARCHAR(4)), 2) + CASE WHEN RTRIM(MaN_TrNSeria) = '' THEN '' ELSE '/' + RTRIM(MaN_TrNSeria) END</t>
+          <t>MaN_TrNRok</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1098,11 +1074,7 @@
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Skróty potwierdzone z obiekty.tsv</t>
-        </is>
-      </c>
+      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1110,29 +1082,35 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MaN_TrNLp</t>
+          <t>MaN_TrNMiesiac</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Kolejność numeru</t>
+          <t>Miesiąc transakcji</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>127, 1, 2</t>
+          <t>3, 5, 6, 11</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Miesiac_Transakcji</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>MaN_TrNMiesiac</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>is_useful=Nie w dokumentacji</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -1141,30 +1119,40 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MaN_KntTyp</t>
+          <t>MaN_TrNSeria</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ID typ kontrahenta</t>
+          <t>Seria dokumentu</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0, 32</t>
+          <t>ZTHKK, SKR, BUS</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Seria</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NULLIF(RTRIM(MaN_TrNSeria), '')</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>GIDTyp — pomocniczy JOIN</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Część Nr_Dokumentu; zachowana osobno</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1172,30 +1160,40 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MaN_KntFirma</t>
+          <t>MaN_TrNNumer</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ID firma kontrahenta</t>
+          <t>Numer transakcji</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0, 1464833</t>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Nr_Dokumentu</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>CASE MaN_GIDTyp WHEN 1089 THEN 'PM' WHEN 1093 THEN 'AWD' WHEN 1601 THEN 'WM' WHEN 1605 THEN 'ZWM' ELSE '??' END + '-' + CAST(MaN_TrNNumer AS VARCHAR(10)) + '/' + RIGHT('0' + CAST(MaN_TrNMiesiac AS VARCHAR(2)), 2) + '/' + RIGHT(CAST(MaN_TrNRok AS VARCHAR(4)), 2) + CASE WHEN RTRIM(MaN_TrNSeria) = '' THEN '' ELSE '/' + RTRIM(MaN_TrNSeria) END</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>GIDFirma — czyste ID systemu</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Skróty z obiekty.tsv</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1203,40 +1201,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MaN_KntNumer</t>
+          <t>MaN_TrNLp</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ID numer kontrahenta</t>
+          <t>Kolejność numeru</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0, 863, 1720</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ID_Kontrahenta</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>CASE WHEN MaN_KntNumer = 0 THEN NULL ELSE MaN_KntNumer END</t>
+          <t>127, 1, 2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Dodać Akronim_Kontrahenta (Knt_Akronim) + Nazwa_Kontrahenta (Knt_Nazwa1) z CDN.KntKarty; LEFT JOIN na KntNumer+KntTyp, warunek KntNumer&gt;0</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1244,17 +1232,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MaN_KntLp</t>
+          <t>MaN_KntTyp</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ID kolejność kontrahenta</t>
+          <t>ID typ kontrahenta</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0, 32</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1264,7 +1252,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>GIDLp — czyste ID systemu</t>
+          <t>GIDTyp — pomocniczy JOIN</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -1275,17 +1263,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MaN_KnATyp</t>
+          <t>MaN_KntFirma</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ID typ adresu kontrahenta</t>
+          <t>ID firma kontrahenta</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0, 864, 896</t>
+          <t>0, 1464833</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1295,7 +1283,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>GIDTyp — pomocniczy JOIN</t>
+          <t>GIDFirma — czyste ID systemu</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -1306,29 +1294,35 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MaN_KnAFirma</t>
+          <t>MaN_KntNumer</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ID firma adresu kontrahenta</t>
+          <t>ID numer kontrahenta</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0, 1464833</t>
+          <t>0, 863, 1720</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ID_Kontrahenta</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_KntNumer = 0 THEN NULL ELSE MaN_KntNumer END</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>GIDFirma — czyste ID systemu</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1337,27 +1331,19 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MaN_KnANumer</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>ID numer adresu kontrahenta</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>0, 276, 862</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>ID_Adresu_Kontrahenta</t>
+          <t>Akronim_Kontrahenta</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_KnANumer = 0 THEN NULL ELSE MaN_KnANumer END</t>
+          <t>LEFT JOIN CDN.KntKarty knt ON knt.Knt_GIDNumer = MaN_KntNumer AND knt.Knt_GIDTyp = MaN_KntTyp AND MaN_KntNumer &gt; 0 › knt.Knt_Akronim</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1368,7 +1354,7 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>FK do adresu dostawy (CDN.KntAdresy?). Czy adres ma kolumnę opisową — weryfikacja INFORMATION_SCHEMA. Jeśli tak — dodać JOIN.</t>
+          <t>JOIN 100% (zweryfikowany)</t>
         </is>
       </c>
     </row>
@@ -1378,29 +1364,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MaN_KnALp</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>ID kolejność adresu kontrahenta</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nazwa_Kontrahenta</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>knt.Knt_Nazwa1</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1409,17 +1393,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MaN_OpeTyp</t>
+          <t>MaN_KntLp</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ID typ operatora</t>
+          <t>ID kolejność kontrahenta</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1429,7 +1413,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>GIDTyp — stały 128 (operator)</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1440,17 +1424,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MaN_OpeFirma</t>
+          <t>MaN_KnATyp</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ID firma operatora</t>
+          <t>ID typ adresu kontrahenta</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1464833</t>
+          <t>0, 864, 896</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1460,7 +1444,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>GIDFirma — czyste ID systemu</t>
+          <t>GIDTyp — pomocniczy JOIN</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -1471,40 +1455,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MaN_OpeNumer</t>
+          <t>MaN_KnAFirma</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ID numer operatora</t>
+          <t>ID firma adresu kontrahenta</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>4, 10, 12, 52, 53</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ID_Operatora</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>MaN_OpeNumer</t>
+          <t>0, 1464833</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Dodać Akronim_Operatora (Ope_Kod) z CDN.OpeKarty</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>GIDFirma — czyste ID systemu</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1512,29 +1486,35 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MaN_OpeLp</t>
+          <t>MaN_KnANumer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ID kolejność operatora</t>
+          <t>ID numer adresu kontrahenta</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0, 276, 862</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ID_Adresu_Kontrahenta</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_KnANumer = 0 THEN NULL ELSE MaN_KnANumer END</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
@@ -1543,30 +1523,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MaN_OpeTypR</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>ID typ operatora (R)</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>0, 128</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Akronim_Adresu_Kontrahenta</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>LEFT JOIN CDN.KntAdresy kna ON kna.KnA_GIDNumer = MaN_KnANumer AND kna.KnA_GIDTyp = MaN_KnATyp AND MaN_KnANumer &gt; 0 › kna.KnA_Akronim</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>GIDTyp — pomocniczy JOIN (0=brak operatora R)</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>CDN.KntAdresy ma KnA_Akronim; JOIN 100% (167232=167232)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1574,17 +1556,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MaN_OpeFirmaR</t>
+          <t>MaN_KnALp</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ID firma operatora (R)</t>
+          <t>ID kolejność adresu kontrahenta</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0, 1464833</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1594,7 +1576,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>GIDFirma — czyste ID systemu</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -1605,40 +1587,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MaN_OpeNumerR</t>
+          <t>MaN_OpeTyp</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ID numer operatora (R)</t>
+          <t>ID typ operatora</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0, 4, 10, 52</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>ID_Operatora_Realizujacego</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>CASE WHEN MaN_OpeNumerR = 0 THEN NULL ELSE MaN_OpeNumerR END</t>
+          <t>128</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Dodać Akronim_Operatora_Realizujacego z CDN.OpeKarty; LEFT JOIN warunek OpeNumerR&gt;0</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>GIDTyp — stały 128 (operator)</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1646,17 +1618,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MaN_OpeLpR</t>
+          <t>MaN_OpeFirma</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ID kolejność operatora (R)</t>
+          <t>ID firma operatora</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1464833</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1666,7 +1638,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>COUNT DISTINCT=1</t>
+          <t>GIDFirma — czyste ID systemu</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
@@ -1677,27 +1649,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MaN_Data3</t>
+          <t>MaN_OpeNumer</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Data wystawienia dokumentu</t>
+          <t>ID numer operatora</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>81237, 81392</t>
+          <t>4, 10, 12, 52, 53</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Data_Wystawienia</t>
+          <t>ID_Operatora</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_Data3 = 0 THEN NULL ELSE CAST(DATEADD(d, MaN_Data3, '18001228') AS DATE) END</t>
+          <t>MaN_OpeNumer</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1706,11 +1678,7 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Clarion DATE</t>
-        </is>
-      </c>
+      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1718,27 +1686,19 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MaN_Stan</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Stan dokumentu</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>0, 1, 2, 5, 6</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Stan_Dokumentu</t>
+          <t>Akronim_Operatora</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>CASE MaN_Stan WHEN 0 THEN 'W edycji' WHEN 1 THEN 'W buforze' WHEN 2 THEN 'Po edycji w buforze' WHEN 5 THEN 'Zatwierdzona' WHEN 6 THEN 'Anulowana' ELSE 'Nieznane (' + CAST(MaN_Stan AS VARCHAR) + ')' END</t>
+          <t>LEFT JOIN CDN.OpeKarty ope ON ope.Ope_GIDNumer = MaN_OpeNumer › ope.Ope_Ident</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1747,7 +1707,11 @@
         </is>
       </c>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>JOIN 100% (zweryfikowany); kolumna Ope_Ident</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1755,12 +1719,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MaN_LicznikKopii</t>
+          <t>MaN_OpeLp</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Licznik kopii</t>
+          <t>ID kolejność operatora</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1775,7 +1739,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
@@ -1786,17 +1750,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MaN_MagDTyp</t>
+          <t>MaN_OpeTypR</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ID typ magazynu docelowego</t>
+          <t>ID typ operatora (R)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>208</t>
+          <t>0, 128</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1806,7 +1770,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>COUNT DISTINCT=1 (stały=208)</t>
+          <t>GIDTyp — pomocniczy JOIN (0=brak operatora R)</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -1817,17 +1781,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MaN_MagDFirma</t>
+          <t>MaN_OpeFirmaR</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ID firma magazynu docelowego</t>
+          <t>ID firma operatora (R)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1464833</t>
+          <t>0, 1464833</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1848,27 +1812,27 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MaN_MagDNumer</t>
+          <t>MaN_OpeNumerR</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ID numer magazynu docelowego</t>
+          <t>ID numer operatora (R)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>1, 5, 7, 8, 9</t>
+          <t>0, 4, 10, 52</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>ID_Magazynu_Docelowego</t>
+          <t>ID_Operatora_Realizujacego</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>MaN_MagDNumer</t>
+          <t>CASE WHEN MaN_OpeNumerR = 0 THEN NULL ELSE MaN_OpeNumerR END</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1877,11 +1841,7 @@
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Dodać Kod_Magazynu_Docelowego (MAG_Kod) + Nazwa_Magazynu_Docelowego (MAG_Nazwa) z CDN.Magazyny</t>
-        </is>
-      </c>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1889,29 +1849,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MaN_MagDLp</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ID kolejność magazynu docelowego</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Akronim_Operatora_Realizujacego</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>LEFT JOIN CDN.OpeKarty ope_r ON ope_r.Ope_GIDNumer = MaN_OpeNumerR AND MaN_OpeNumerR &gt; 0 › ope_r.Ope_Ident</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1920,40 +1878,30 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MaN_FrsID</t>
+          <t>MaN_OpeLpR</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ID centrum struktury praw</t>
+          <t>ID kolejność operatora (R)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>1, 6, 8, 11, 38, 39</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>ID_Centrum</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>MaN_FrsID</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Dodać Nazwa_Centrum (FRS_Nazwa) z CDN.FrmStruktura ON FRS_ID</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>COUNT DISTINCT=1</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1961,30 +1909,40 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MaN_Aktywny</t>
+          <t>MaN_Data3</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Aktywny (flaga)</t>
+          <t>Data wystawienia dokumentu</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>0, 84, 29740</t>
+          <t>81237, 81392</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Data_Wystawienia</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_Data3 = 0 THEN NULL ELSE CAST(DATEADD(d, MaN_Data3, '18001228') AS DATE) END</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>is_useful=Nie w dokumentacji</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Clarion DATE</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1992,29 +1950,35 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MaN_Wsk</t>
+          <t>MaN_Stan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Wskaźnik zaznaczenia</t>
+          <t>Stan dokumentu</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0, 1, 2, 3</t>
+          <t>0, 1, 2, 5, 6</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Stan_Dokumentu</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>CASE MaN_Stan WHEN 0 THEN 'W edycji' WHEN 1 THEN 'W buforze' WHEN 2 THEN 'Po edycji w buforze' WHEN 5 THEN 'Zatwierdzona' WHEN 6 THEN 'Anulowana' ELSE 'Nieznane (' + CAST(MaN_Stan AS VARCHAR) + ')' END</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>is_useful=Nie w dokumentacji</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
@@ -2023,35 +1987,29 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MaN_CechaOpis</t>
+          <t>MaN_LicznikKopii</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Cecha transakcji</t>
+          <t>Licznik kopii</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Wzory, SEZON, Uszkodzenie</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>Cecha</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>MaN_CechaOpis</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
       <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
@@ -2060,17 +2018,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MaN_OpeTypM</t>
+          <t>MaN_MagDTyp</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ID typ operatora modyfikującego</t>
+          <t>ID typ magazynu docelowego</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>208</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2080,7 +2038,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>GIDTyp — pomocniczy JOIN</t>
+          <t>COUNT DISTINCT=1 (stały=208)</t>
         </is>
       </c>
       <c r="I47" t="inlineStr"/>
@@ -2091,12 +2049,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MaN_OpeFirmaM</t>
+          <t>MaN_MagDFirma</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ID firma operatora modyfikującego</t>
+          <t>ID firma magazynu docelowego</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2122,27 +2080,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MaN_OpeNumerM</t>
+          <t>MaN_MagDNumer</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ID numer operatora modyfikującego</t>
+          <t>ID numer magazynu docelowego</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2, 4, 10, 52</t>
+          <t>1, 5, 7, 8, 9</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>ID_Operatora_Modyfikujacego</t>
+          <t>ID_Magazynu_Docelowego</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_OpeNumerM = 0 THEN NULL ELSE MaN_OpeNumerM END</t>
+          <t>MaN_MagDNumer</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2151,11 +2109,7 @@
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Dodać Akronim_Operatora_Modyfikujacego z CDN.OpeKarty; LEFT JOIN warunek OpeNumerM&gt;0</t>
-        </is>
-      </c>
+      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2163,30 +2117,32 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MaN_OpeLpM</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>ID kolejność operatora modyfikującego</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Kod_Magazynu_Docelowego</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>LEFT JOIN CDN.Magazyny mag_d ON mag_d.MAG_GIDNumer = MaN_MagDNumer › mag_d.MAG_Kod</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>COUNT DISTINCT=1</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>JOIN 100% (zweryfikowany)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2194,29 +2150,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MaN_ZaNTyp</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>ID typ nagłówka zamówienia</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>0, 960</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Nazwa_Magazynu_Docelowego</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>mag_d.MAG_Nazwa</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>GIDTyp — pomocniczy JOIN</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
@@ -2225,17 +2179,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MaN_ZaNFirma</t>
+          <t>MaN_MagDLp</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ID firma nagłówka zamówienia</t>
+          <t>ID kolejność magazynu docelowego</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>0, 1464833</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2245,7 +2199,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>GIDFirma — czyste ID systemu</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I52" t="inlineStr"/>
@@ -2256,27 +2210,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MaN_ZaNNumer</t>
+          <t>MaN_FrsID</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ID numer nagłówka zamówienia</t>
+          <t>ID centrum struktury praw</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>0, 807, 892, 2546</t>
+          <t>1, 6, 8, 11, 38, 39</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ID_Zamowienia</t>
+          <t>ID_Centrum</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_ZaNNumer = 0 THEN NULL ELSE MaN_ZaNNumer END</t>
+          <t>MaN_FrsID</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2293,30 +2247,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MaN_ZaNLp</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>ID kolejność nagłówka zamówienia</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>0</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Nazwa_Centrum</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>LEFT JOIN CDN.FrmStruktura frs ON frs.FRS_ID = MaN_FrsID › frs.FRS_Nazwa</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>JOIN 100% (zweryfikowany)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2324,17 +2280,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MaN_TypZrd</t>
+          <t>MaN_Aktywny</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Typ dokumentu źródłowego zlecenia</t>
+          <t>Aktywny (flaga)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0, 84, 29740</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2344,7 +2300,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>COUNT DISTINCT=1</t>
+          <t>is_useful=Nie w dokumentacji</t>
         </is>
       </c>
       <c r="I55" t="inlineStr"/>
@@ -2355,17 +2311,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MaN_RokMiesiac</t>
+          <t>MaN_Wsk</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>RokMiesiąc (z Data3)</t>
+          <t>Wskaźnik zaznaczenia</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>202311, 202305</t>
+          <t>0, 1, 2, 3</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2375,7 +2331,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Redundantne — wyliczalne z Data_Wystawienia</t>
+          <t>is_useful=Nie w dokumentacji</t>
         </is>
       </c>
       <c r="I56" t="inlineStr"/>
@@ -2386,29 +2342,35 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MaN_FrmNumer</t>
+          <t>MaN_CechaOpis</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Numer pieczątki</t>
+          <t>Cecha transakcji</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Wzory, SEZON, Uszkodzenie</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Cecha</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>MaN_CechaOpis</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>is_useful=Nie w dokumentacji</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2417,15 +2379,19 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MaN_ZewnetrznySys</t>
+          <t>MaN_OpeTypM</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ID systemu zewnętrznego</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
+          <t>ID typ operatora modyfikującego</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
           <t>Nie</t>
@@ -2433,7 +2399,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>GIDTyp — pomocniczy JOIN</t>
         </is>
       </c>
       <c r="I58" t="inlineStr"/>
@@ -2444,15 +2410,19 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MaN_ZewnetrzneId</t>
+          <t>MaN_OpeFirmaM</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ID dokumentu w systemie zewnętrznym</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr"/>
+          <t>ID firma operatora modyfikującego</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1464833</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr">
         <is>
           <t>Nie</t>
@@ -2460,7 +2430,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>GIDFirma — czyste ID systemu</t>
         </is>
       </c>
       <c r="I59" t="inlineStr"/>
@@ -2471,27 +2441,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MaN_LastMod</t>
+          <t>MaN_OpeNumerM</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Czas ostatniej modyfikacji (TS)</t>
+          <t>ID numer operatora modyfikującego</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>1054293279</t>
+          <t>2, 4, 10, 52</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>DataCzas_Modyfikacji</t>
+          <t>ID_Operatora_Modyfikujacego</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_LastMod = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_LastMod, '1990-01-01') AS DATETIME) END</t>
+          <t>CASE WHEN MaN_OpeNumerM = 0 THEN NULL ELSE MaN_OpeNumerM END</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2500,11 +2470,7 @@
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Clarion TIMESTAMP</t>
-        </is>
-      </c>
+      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2512,27 +2478,19 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MaN_DataOd</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Data/czas rozpoczęcia</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>1054252800</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
-          <t>DataCzas_Od</t>
+          <t>Akronim_Operatora_Modyfikujacego</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_DataOd = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_DataOd, '1990-01-01') AS DATETIME) END</t>
+          <t>LEFT JOIN CDN.OpeKarty ope_m ON ope_m.Ope_GIDNumer = MaN_OpeNumerM AND MaN_OpeNumerM &gt; 0 › ope_m.Ope_Ident</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2541,11 +2499,7 @@
         </is>
       </c>
       <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Clarion TIMESTAMP — data/godzina przyjęcia/wydania</t>
-        </is>
-      </c>
+      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2553,40 +2507,30 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MaN_DataDo</t>
+          <t>MaN_OpeLpM</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Data/czas zakończenia</t>
+          <t>ID kolejność operatora modyfikującego</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1054339140</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>DataCzas_Do</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>CASE WHEN MaN_DataDo = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_DataDo, '1990-01-01') AS DATETIME) END</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Clarion TIMESTAMP — data/godzina przyjęcia/wydania</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>COUNT DISTINCT=1</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2594,15 +2538,19 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MaN_SpeTyp</t>
+          <t>MaN_ZaNTyp</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ID typ spedytora</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
+          <t>ID typ nagłówka zamówienia</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0, 960</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr">
         <is>
           <t>Nie</t>
@@ -2610,7 +2558,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>GIDTyp — pomocniczy JOIN</t>
         </is>
       </c>
       <c r="I63" t="inlineStr"/>
@@ -2621,15 +2569,19 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MaN_SpeFirma</t>
+          <t>MaN_ZaNFirma</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ID firma spedytora</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
+          <t>ID firma nagłówka zamówienia</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>0, 1464833</t>
+        </is>
+      </c>
       <c r="G64" t="inlineStr">
         <is>
           <t>Nie</t>
@@ -2648,25 +2600,35 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MaN_SpeNumer</t>
+          <t>MaN_ZaNNumer</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>ID numer spedytora</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
+          <t>ID numer nagłówka zamówienia</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0, 807, 892, 2546</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>ID_Zamowienia</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_ZaNNumer = 0 THEN NULL ELSE MaN_ZaNNumer END</t>
+        </is>
+      </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>COUNT DISTINCT=1</t>
-        </is>
-      </c>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
@@ -2675,26 +2637,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MaN_SpeLp</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>ID kolejność spedytora</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
       <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Nr_Zamowienia</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>LEFT JOIN CDN.ZamNag zan ON zan.ZaN_GIDNumer = MaN_ZaNNumer AND MaN_ZaNNumer &gt; 0; CASE WHEN MaN_ZaNNumer = 0 THEN NULL ELSE CASE zan.ZaN_ZamTyp WHEN 640 THEN 'OFZ' WHEN 768 THEN 'OFS' WHEN 1152 THEN 'ZZ' WHEN 1280 THEN 'ZS' WHEN 2688 THEN 'ZZ' WHEN 2816 THEN 'ZS' ELSE '??' END + '-' + CAST(zan.ZaN_ZamNumer AS VARCHAR(10)) + '/' + RIGHT('0' + CAST(zan.ZaN_ZamMiesiac AS VARCHAR(2)), 2) + '/' + RIGHT(CAST(zan.ZaN_ZamRok AS VARCHAR(4)), 2) + CASE WHEN RTRIM(zan.ZaN_ZamSeria) = '' THEN '' ELSE '/' + RTRIM(zan.ZaN_ZamSeria) END END</t>
+        </is>
+      </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>GIDLp — czyste ID systemu</t>
-        </is>
-      </c>
-      <c r="I66" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>JOIN 100% (10315=10315); prefiks z CASE zan.ZaN_ZamTyp — analogicznie do ZamNag</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2702,15 +2670,19 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MaN_TrasaId</t>
+          <t>MaN_ZaNLp</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ID trasy</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
+          <t>ID kolejność nagłówka zamówienia</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>Nie</t>
@@ -2718,7 +2690,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>COUNT DISTINCT=1</t>
+          <t>GIDLp — czyste ID systemu</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -2729,35 +2701,29 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MaN_Realizacja</t>
+          <t>MaN_TypZrd</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Realizacja (%)</t>
+          <t>Typ dokumentu źródłowego zlecenia</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>0, 100</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Realizacja_Procent</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>MaN_Realizacja</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>COUNT DISTINCT=1</t>
+        </is>
+      </c>
       <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
@@ -2766,35 +2732,29 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MaN_SposobDostawy</t>
+          <t>MaN_RokMiesiac</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sposób dostawy</t>
+          <t>RokMiesiąc (z Data3)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Geodis, Pocztex, DHL</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Sposob_Dostawy</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>MaN_SposobDostawy</t>
+          <t>202311, 202305</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H69" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Redundantne — wyliczalne z Data_Wystawienia</t>
+        </is>
+      </c>
       <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
@@ -2803,40 +2763,30 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MaN_Priorytet</t>
+          <t>MaN_FrmNumer</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Priorytet zlecenia</t>
+          <t>Numer pieczątki</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>0, 20, 30</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Priorytet_Zlecenia</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>MaN_Priorytet</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Wartości 0/20/30 — brak opisu w dokumentacji. Czy znane znaczenie? Jeśli tak — dodać CASE</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2844,35 +2794,25 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MaN_Status</t>
+          <t>MaN_ZewnetrznySys</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Status zlecenia</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>0, 1, 4, 5</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Status_Zlecenia</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>CASE MaN_Status WHEN 0 THEN 'Niezatwierdzony' WHEN 1 THEN 'Zatwierdzony' WHEN 2 THEN 'W realizacji' WHEN 3 THEN 'Zrealizowany' WHEN 4 THEN 'Zamknięty' WHEN 5 THEN 'Zamknięty bez realizacji' WHEN 6 THEN 'Zamknięty do edycji' ELSE 'Nieznane (' + CAST(MaN_Status AS VARCHAR) + ')' END</t>
-        </is>
-      </c>
+          <t>ID systemu zewnętrznego</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr"/>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
       <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
@@ -2881,40 +2821,26 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MaN_WMS</t>
+          <t>MaN_ZewnetrzneId</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Dokument w WMS (flaga)</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>0, 177</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Dokument_WMS</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>CASE MaN_WMS WHEN 0 THEN 'Nie' WHEN 177 THEN 'Tak' ELSE 'Nieznane (' + CAST(MaN_WMS AS VARCHAR) + ')' END</t>
-        </is>
-      </c>
+          <t>ID dokumentu w systemie zewnętrznym</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Tak</t>
-        </is>
-      </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Wartość 177 = WMS (jedyna wartość niezerowa w danych)</t>
-        </is>
-      </c>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2922,27 +2848,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MaN_DataZatwierdzenia</t>
+          <t>MaN_LastMod</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Data zatwierdzenia/zamknięcia</t>
+          <t>Czas ostatniej modyfikacji (TS)</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>0, 81376, 81392</t>
+          <t>1054293279</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Data_Zatwierdzenia</t>
+          <t>DataCzas_Modyfikacji</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>CASE WHEN MaN_DataZatwierdzenia = 0 THEN NULL ELSE CAST(DATEADD(d, MaN_DataZatwierdzenia, '18001228') AS DATE) END</t>
+          <t>CASE WHEN MaN_LastMod = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_LastMod, '1990-01-01') AS DATETIME) END</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2953,7 +2879,7 @@
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr">
         <is>
-          <t>Clarion DATE</t>
+          <t>Clarion TIMESTAMP</t>
         </is>
       </c>
     </row>
@@ -2963,27 +2889,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MaN_Zrodlo</t>
+          <t>MaN_DataOd</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Powiązanie z dokumentem źródłowym</t>
+          <t>Data/czas rozpoczęcia</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>0, 1</t>
+          <t>1054252800</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Powiazanie_Zrodlowe</t>
+          <t>DataCzas_Od</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>CASE MaN_Zrodlo WHEN 0 THEN 'Niepowiązany' WHEN 1 THEN 'Powiązany' WHEN 2 THEN 'Powiązany wielokrotnie' ELSE 'Nieznane (' + CAST(MaN_Zrodlo AS VARCHAR) + ')' END</t>
+          <t>CASE WHEN MaN_DataOd = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_DataOd, '1990-01-01') AS DATETIME) END</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2992,7 +2918,11 @@
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Clarion TIMESTAMP</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3000,26 +2930,40 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MaN_RezerwujZasoby</t>
+          <t>MaN_DataDo</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Rezerwuj zasoby (WMS)</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
+          <t>Data/czas zakończenia</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>1054339140</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>DataCzas_Do</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_DataDo = 0 THEN NULL ELSE CAST(DATEADD(ss, MaN_DataDo, '1990-01-01') AS DATETIME) END</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Nie</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>is_useful=Nie w dokumentacji</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr"/>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Clarion TIMESTAMP</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3027,12 +2971,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MaN_WMSDokWewn</t>
+          <t>MaN_SpeTyp</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Wystawianie dok. WMS dla MMW/MMP</t>
+          <t>ID typ spedytora</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -3054,12 +2998,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MaN_WZWMPelneJPom</t>
+          <t>MaN_SpeFirma</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Wymuś pełne ilości w J.pom.</t>
+          <t>ID firma spedytora</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -3070,7 +3014,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>GIDFirma — czyste ID systemu</t>
         </is>
       </c>
       <c r="I77" t="inlineStr"/>
@@ -3081,12 +3025,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MaN_KolejnoscZal</t>
+          <t>MaN_SpeNumer</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Kolejność załadunku</t>
+          <t>ID numer spedytora</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -3097,7 +3041,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>is_useful=Nie w dokumentacji</t>
+          <t>COUNT DISTINCT=1</t>
         </is>
       </c>
       <c r="I78" t="inlineStr"/>
@@ -3108,12 +3052,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MaN_LaczPozycje</t>
+          <t>MaN_SpeLp</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Agregacja pozycji w partii</t>
+          <t>ID kolejność spedytora</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -3124,10 +3068,443 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
+          <t>GIDLp — czyste ID systemu</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MaN_TrasaId</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ID trasy</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>COUNT DISTINCT=1</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>MaN_Realizacja</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Realizacja (%)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>0, 100</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Realizacja_Procent</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>MaN_Realizacja</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MaN_SposobDostawy</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sposób dostawy</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Geodis, Pocztex, DHL</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Sposob_Dostawy</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>MaN_SposobDostawy</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MaN_Priorytet</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Priorytet zlecenia</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>0, 20, 30</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Priorytet_Zlecenia</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>MaN_Priorytet</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Wartości 0/20/30 — brak opisu w dokumentacji. Pytanie do użytkownika: czy znane znaczenie?</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MaN_Status</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Status zlecenia</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>0, 1, 4, 5</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Status_Zlecenia</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>CASE MaN_Status WHEN 0 THEN 'Niezatwierdzony' WHEN 1 THEN 'Zatwierdzony' WHEN 2 THEN 'W realizacji' WHEN 3 THEN 'Zrealizowany' WHEN 4 THEN 'Zamknięty' WHEN 5 THEN 'Zamknięty bez realizacji' WHEN 6 THEN 'Zamknięty do edycji' ELSE 'Nieznane (' + CAST(MaN_Status AS VARCHAR) + ')' END</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>MaN_WMS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Dokument w WMS (flaga)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>0, 177</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Dokument_WMS</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>CASE MaN_WMS WHEN 0 THEN 'Nie' WHEN 177 THEN 'Tak' ELSE 'Nieznane (' + CAST(MaN_WMS AS VARCHAR) + ')' END</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Wartość 177 = WMS (jedyna niezerowa w danych)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MaN_DataZatwierdzenia</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Data zatwierdzenia/zamknięcia</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>0, 81376, 81392</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Data_Zatwierdzenia</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>CASE WHEN MaN_DataZatwierdzenia = 0 THEN NULL ELSE CAST(DATEADD(d, MaN_DataZatwierdzenia, '18001228') AS DATE) END</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Clarion DATE</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MaN_Zrodlo</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Powiązanie z dokumentem źródłowym</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>0, 1</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Powiazanie_Zrodlowe</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>CASE MaN_Zrodlo WHEN 0 THEN 'Niepowiązany' WHEN 1 THEN 'Powiązany' WHEN 2 THEN 'Powiązany wielokrotnie' ELSE 'Nieznane (' + CAST(MaN_Zrodlo AS VARCHAR) + ')' END</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Tak</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MaN_RezerwujZasoby</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Rezerwuj zasoby (WMS)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
           <t>is_useful=Nie w dokumentacji</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
+      <c r="I88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MaN_WMSDokWewn</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Wystawianie dok. WMS dla MMW/MMP</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MaN_WZWMPelneJPom</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Wymuś pełne ilości w J.pom.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MaN_KolejnoscZal</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Kolejność załadunku</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>MaN_LaczPozycje</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Agregacja pozycji w partii</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Nie</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>is_useful=Nie w dokumentacji</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>